<commit_message>
v2.7.6: 美团 LongCat 每日免费额度入流(560B Flash-Chat,OpenAI/Anthropic双兼容,数额待实锤补daily_wun)
</commit_message>
<xml_diff>
--- a/data-research/信息源总表-全量版.xlsx
+++ b/data-research/信息源总表-全量版.xlsx
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4354,6 +4354,58 @@
       <c r="J85" t="inlineStr">
         <is>
           <t>聚合平台类（中间商层在收录范围内）</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>线索-套餐(海外)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>z.ai GLM Coding Plan 海外版</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://z.ai</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>套餐订阅</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>⏳ 主管核实</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Reddit+第三方</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Lite$18/Pro$80/Max$168；配额≈Claude同级3倍；海外ZCode $16.2/月</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>⌨️Coding面板海外版候选；无常驻免费额度</t>
         </is>
       </c>
     </row>
@@ -5432,7 +5484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6140,6 +6192,28 @@
         </is>
       </c>
       <c r="D32" t="inlineStr">
+        <is>
+          <t>总表</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>z.ai 海外 Coding Plan 查实（三档价格+3倍配额定位）→⌨️Coding面板海外版候选</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>15分钟找源巡检</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>总表</t>
         </is>

</xml_diff>

<commit_message>
v2.9.4: 海外聚合商专项信源组(老板指令)——OpenRouter/OpenCode/Kilo/OmniRoute/TaoToken/llm7/Agnes/Regolo/TokenHarbor/IteraCompute/Upstage/Fireworks/Replicate/HF/Together/Groq 16源 lane=ov-aggregator 入采集器(现役97),reseller导航补6站,Excel加专项sheet
</commit_message>
<xml_diff>
--- a/data-research/信息源总表-全量版.xlsx
+++ b/data-research/信息源总表-全量版.xlsx
@@ -13,6 +13,7 @@
     <sheet name="发现日志" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="候选源池" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="长期源清单" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="海外聚合专项" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67732,4 +67733,375 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>盯防重点</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>lane</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>收录时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ov-kilo-pricing</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kilo Code</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://kilo.ai/pricing</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ov-taotoken</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TaoToken 聚合网关</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://taotoken.net</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ov-llm7-docs</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>llm7 免费聚合</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://docs.llm7.io</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ov-agnes-ai</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Agnes AI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://platform.agnes-ai.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ov-regolo-pricing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Regolo.ai</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://regolo.ai/pricing/</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ov-tokenharbor</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TokenHarbor</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://tokenharbor.ai/pricing</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ov-iteracompute</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IteraCompute</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://platform.iteracompute.com/api-keys</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ov-upstage</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Upstage</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://console.upstage.ai</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ov-replicate-pricing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Replicate</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://replicate.com/pricing</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ov-hf-inference</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HuggingFace 推理</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/docs/inference-providers/index</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>免费层/credits/限额变动</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ov-aggregator</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v2.11.0: 整站彻底 SEO(老板指令'qa啥的都搞，Google 可收录')——①head 强化: title/desc/keywords 重写+OG 全套+Twitter Card+RSS alternate+preconnect;②结构化数据: WebSite+Organization+FAQPage(8 问与可见 FAQ 同步)+guides Article JSON-LD;③FAQ 区块 8 条(details 折叠,含'DS Flash 等效/收益算法/最大额度平台/可信度/比价器'关键词);④noscript 静态兜底(无 JS 爬虫可读核心情报+攻略链接);⑤h1 补齐(logo span→h1);⑥sitemap 全量 12 URL(首页+10 攻略+rss,lastmod 今日);⑦guides 模板补 meta description/canonical/og/Article JSON-LD 重建 10 篇;⑧0 万口径修复: 无数额条目显示'免费·额度未公布'不再误导;JSC 语法门+JSON-LD 校验+浏览器实测(rows 46/FAQ 8/h1 ✓)
</commit_message>
<xml_diff>
--- a/data-research/信息源总表-全量版.xlsx
+++ b/data-research/信息源总表-全量版.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K138"/>
+  <dimension ref="A1:K141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7493,6 +7493,158 @@
           <t>新子类候选</t>
         </is>
       </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>线索-活动(雷达)⭐</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>「白捡价值900块的大模型额度」长文+领取指南内容潮</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>(公众号多帖)</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>活动聚合</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>⏳ 主管核实(高优)</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>多帖内容潮</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>小米MiMo入口/双11券+AI额度15条/现在能领清单——1111预热实锤；长文可解析直达全文提取清单</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>雷达轮34</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>情报-生态(TG雷达)</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>GitHub 发布 Copilot Fusion 多模型自动编排</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>(TG AI_News_CN·Universe2026)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>生态</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>⏳ 主管核实</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>官方大会</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>自动路由 OpenAI/Anthropic/Google——⌨️Coding面板相关新品</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>TG监视器首捕</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>情报-成本(TG雷达)</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Particle-1(DeepSeek V4.1 Flash后训练)编码token用量-39%</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>(TG AI_News_CN)</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>成本优化</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>👁 观察</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>实测基准</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>88个Go任务实测：token-39%/成本降低</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10585,7 +10737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12109,6 +12261,50 @@
       <c r="D69" t="inlineStr">
         <is>
           <t>日志</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>⭐雷达轮34：「白捡900块额度」长文+领取指南内容潮（1111预热实锤）；Trae国际站源(主会话)；垃圾账号清理+提取加固</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>公众号专属管线</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>总表</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>⭐Telegram监视器收编4频道(linuxdoit/linuxdo_tg/AI_Copilot/AI_News_CN)首扫11命中：Copilot Fusion发布+Particle-1省token实测+Anthropic企业管控</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>TG管线</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>总表</t>
         </is>
       </c>
     </row>

</xml_diff>